<commit_message>
Final ACC II paper modeling
</commit_message>
<xml_diff>
--- a/InputData/trans/VSbS/Vehicle Shares by Subregion.xlsx
+++ b/InputData/trans/VSbS/Vehicle Shares by Subregion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jeff Rissman\CodeRepositories\eps-us\InputData\trans\VSbS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-maryland\InputData\trans\VSbS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7C4D67-74A1-4BF9-A001-F474636F2E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF230E39-7A45-46E2-9F8D-6933CEE91E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16440" yWindow="2445" windowWidth="29940" windowHeight="20805" xr2:uid="{F34BB550-7D2B-439D-9C81-D72ED5B29ABD}"/>
+    <workbookView xWindow="29745" yWindow="3540" windowWidth="17505" windowHeight="9735" activeTab="1" xr2:uid="{F34BB550-7D2B-439D-9C81-D72ED5B29ABD}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="159">
   <si>
     <t>VSbS Vehicle Shares by Subregion</t>
   </si>
@@ -380,6 +380,159 @@
   </si>
   <si>
     <t>U.S. Data Notes</t>
+  </si>
+  <si>
+    <t>subregion1</t>
+  </si>
+  <si>
+    <t>subregion2</t>
+  </si>
+  <si>
+    <t>subregion3</t>
+  </si>
+  <si>
+    <t>subregion4</t>
+  </si>
+  <si>
+    <t>subregion5</t>
+  </si>
+  <si>
+    <t>subregion6</t>
+  </si>
+  <si>
+    <t>subregion7</t>
+  </si>
+  <si>
+    <t>subregion8</t>
+  </si>
+  <si>
+    <t>subregion9</t>
+  </si>
+  <si>
+    <t>subregion10</t>
+  </si>
+  <si>
+    <t>subregion11</t>
+  </si>
+  <si>
+    <t>subregion12</t>
+  </si>
+  <si>
+    <t>subregion13</t>
+  </si>
+  <si>
+    <t>subregion14</t>
+  </si>
+  <si>
+    <t>subregion15</t>
+  </si>
+  <si>
+    <t>subregion16</t>
+  </si>
+  <si>
+    <t>subregion17</t>
+  </si>
+  <si>
+    <t>subregion18</t>
+  </si>
+  <si>
+    <t>subregion19</t>
+  </si>
+  <si>
+    <t>subregion20</t>
+  </si>
+  <si>
+    <t>subregion21</t>
+  </si>
+  <si>
+    <t>subregion22</t>
+  </si>
+  <si>
+    <t>subregion23</t>
+  </si>
+  <si>
+    <t>subregion24</t>
+  </si>
+  <si>
+    <t>subregion25</t>
+  </si>
+  <si>
+    <t>subregion26</t>
+  </si>
+  <si>
+    <t>subregion27</t>
+  </si>
+  <si>
+    <t>subregion28</t>
+  </si>
+  <si>
+    <t>subregion29</t>
+  </si>
+  <si>
+    <t>subregion30</t>
+  </si>
+  <si>
+    <t>subregion31</t>
+  </si>
+  <si>
+    <t>subregion32</t>
+  </si>
+  <si>
+    <t>subregion33</t>
+  </si>
+  <si>
+    <t>subregion34</t>
+  </si>
+  <si>
+    <t>subregion35</t>
+  </si>
+  <si>
+    <t>subregion36</t>
+  </si>
+  <si>
+    <t>subregion37</t>
+  </si>
+  <si>
+    <t>subregion38</t>
+  </si>
+  <si>
+    <t>subregion39</t>
+  </si>
+  <si>
+    <t>subregion40</t>
+  </si>
+  <si>
+    <t>subregion41</t>
+  </si>
+  <si>
+    <t>subregion42</t>
+  </si>
+  <si>
+    <t>subregion43</t>
+  </si>
+  <si>
+    <t>subregion44</t>
+  </si>
+  <si>
+    <t>subregion45</t>
+  </si>
+  <si>
+    <t>subregion46</t>
+  </si>
+  <si>
+    <t>subregion47</t>
+  </si>
+  <si>
+    <t>subregion48</t>
+  </si>
+  <si>
+    <t>subregion49</t>
+  </si>
+  <si>
+    <t>subregion50</t>
+  </si>
+  <si>
+    <t>subregion51</t>
   </si>
 </sst>
 </file>
@@ -1075,7 +1228,7 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="37" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
@@ -1244,6 +1397,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1274,11 +1429,6 @@
     <xf numFmtId="37" fontId="5" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Comma 2" xfId="5" xr:uid="{7B2DBB66-964B-4992-8A85-CF7563C0181E}"/>
@@ -1771,9 +1921,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30B0F8C0-DE1A-4000-9351-A11EE8CD5BC4}">
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="70.140625" customWidth="1"/>
+    <col min="2" max="2" width="70.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1815,26 +1965,23 @@
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="112" t="s">
+      <c r="A10" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="112" t="s">
+      <c r="A11" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="112"/>
-    </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="113" t="s">
+      <c r="A13" s="102" t="s">
         <v>107</v>
       </c>
-      <c r="B13" s="114"/>
-    </row>
-    <row r="14" spans="1:2" s="116" customFormat="1">
-      <c r="A14" s="115"/>
+      <c r="B13" s="103"/>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="1"/>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
@@ -1894,32 +2041,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{949F6402-DD66-4CAC-8910-748EA4AEB83B}">
   <dimension ref="A1:P63"/>
-  <sheetFormatPr defaultRowHeight="8.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="8"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" style="4" customWidth="1"/>
-    <col min="2" max="16" width="9.85546875" style="4" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="11.26953125" style="4" customWidth="1"/>
+    <col min="2" max="16" width="9.81640625" style="4" customWidth="1"/>
+    <col min="17" max="16384" width="9.1796875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15">
-      <c r="A1" s="103" t="s">
+    <row r="1" spans="1:16" ht="14">
+      <c r="A1" s="105" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="103"/>
-      <c r="C1" s="103"/>
-      <c r="D1" s="103"/>
-      <c r="E1" s="103"/>
-      <c r="F1" s="103"/>
-      <c r="G1" s="103"/>
-      <c r="H1" s="103"/>
-      <c r="I1" s="103"/>
-      <c r="J1" s="103"/>
-      <c r="K1" s="103"/>
-      <c r="L1" s="103"/>
-      <c r="M1" s="103"/>
-      <c r="N1" s="103"/>
-      <c r="O1" s="103"/>
-      <c r="P1" s="103"/>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
+      <c r="K1" s="105"/>
+      <c r="L1" s="105"/>
+      <c r="M1" s="105"/>
+      <c r="N1" s="105"/>
+      <c r="O1" s="105"/>
+      <c r="P1" s="105"/>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" s="98"/>
@@ -1963,51 +2110,51 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="94"/>
-      <c r="B4" s="104" t="s">
+      <c r="B4" s="106" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="105"/>
-      <c r="D4" s="105"/>
-      <c r="E4" s="105"/>
-      <c r="F4" s="105"/>
-      <c r="G4" s="105"/>
-      <c r="H4" s="105"/>
-      <c r="I4" s="105"/>
-      <c r="J4" s="105"/>
-      <c r="K4" s="105"/>
-      <c r="L4" s="105"/>
-      <c r="M4" s="105"/>
-      <c r="N4" s="105"/>
-      <c r="O4" s="105"/>
-      <c r="P4" s="106"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="107"/>
+      <c r="E4" s="107"/>
+      <c r="F4" s="107"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="107"/>
+      <c r="I4" s="107"/>
+      <c r="J4" s="107"/>
+      <c r="K4" s="107"/>
+      <c r="L4" s="107"/>
+      <c r="M4" s="107"/>
+      <c r="N4" s="107"/>
+      <c r="O4" s="107"/>
+      <c r="P4" s="108"/>
     </row>
     <row r="5" spans="1:16" ht="9">
       <c r="A5" s="79"/>
-      <c r="B5" s="107" t="s">
+      <c r="B5" s="109" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="109" t="s">
+      <c r="C5" s="110"/>
+      <c r="D5" s="110"/>
+      <c r="E5" s="111" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="108"/>
-      <c r="G5" s="110"/>
-      <c r="H5" s="108" t="s">
+      <c r="F5" s="110"/>
+      <c r="G5" s="112"/>
+      <c r="H5" s="110" t="s">
         <v>71</v>
       </c>
-      <c r="I5" s="108"/>
-      <c r="J5" s="108"/>
-      <c r="K5" s="109" t="s">
+      <c r="I5" s="110"/>
+      <c r="J5" s="110"/>
+      <c r="K5" s="111" t="s">
         <v>70</v>
       </c>
-      <c r="L5" s="108"/>
-      <c r="M5" s="110"/>
-      <c r="N5" s="108" t="s">
+      <c r="L5" s="110"/>
+      <c r="M5" s="112"/>
+      <c r="N5" s="110" t="s">
         <v>69</v>
       </c>
-      <c r="O5" s="108"/>
-      <c r="P5" s="111"/>
+      <c r="O5" s="110"/>
+      <c r="P5" s="113"/>
     </row>
     <row r="6" spans="1:16" ht="9">
       <c r="A6" s="79" t="s">
@@ -4789,25 +4936,25 @@
       <c r="O62" s="5"/>
       <c r="P62" s="5"/>
     </row>
-    <row r="63" spans="1:16" ht="39.6" customHeight="1">
-      <c r="A63" s="102" t="s">
+    <row r="63" spans="1:16" ht="39.65" customHeight="1">
+      <c r="A63" s="104" t="s">
         <v>6</v>
       </c>
-      <c r="B63" s="102"/>
-      <c r="C63" s="102"/>
-      <c r="D63" s="102"/>
-      <c r="E63" s="102"/>
-      <c r="F63" s="102"/>
-      <c r="G63" s="102"/>
-      <c r="H63" s="102"/>
-      <c r="I63" s="102"/>
-      <c r="J63" s="102"/>
-      <c r="K63" s="102"/>
-      <c r="L63" s="102"/>
-      <c r="M63" s="102"/>
-      <c r="N63" s="102"/>
-      <c r="O63" s="102"/>
-      <c r="P63" s="102"/>
+      <c r="B63" s="104"/>
+      <c r="C63" s="104"/>
+      <c r="D63" s="104"/>
+      <c r="E63" s="104"/>
+      <c r="F63" s="104"/>
+      <c r="G63" s="104"/>
+      <c r="H63" s="104"/>
+      <c r="I63" s="104"/>
+      <c r="J63" s="104"/>
+      <c r="K63" s="104"/>
+      <c r="L63" s="104"/>
+      <c r="M63" s="104"/>
+      <c r="N63" s="104"/>
+      <c r="O63" s="104"/>
+      <c r="P63" s="104"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5001,10 +5148,10 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:G61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="7" width="13.7109375" customWidth="1"/>
+    <col min="2" max="7" width="13.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5032,11 +5179,10 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="B2">
-        <f>'Table MV-1'!D10/'Table MV-1'!$D$61</f>
-        <v>1.9359587122498342E-2</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <f>'Table MV-1'!G10/'Table MV-1'!$G$61</f>
@@ -5058,11 +5204,10 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>109</v>
       </c>
       <c r="B3">
-        <f>'Table MV-1'!D11/'Table MV-1'!$D$61</f>
-        <v>1.6278452622477892E-3</v>
+        <v>0</v>
       </c>
       <c r="C3">
         <f>'Table MV-1'!G11/'Table MV-1'!$G$61</f>
@@ -5084,11 +5229,10 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>110</v>
       </c>
       <c r="B4">
-        <f>'Table MV-1'!D12/'Table MV-1'!$D$61</f>
-        <v>2.2923014439488926E-2</v>
+        <v>0</v>
       </c>
       <c r="C4">
         <f>'Table MV-1'!G12/'Table MV-1'!$G$61</f>
@@ -5110,11 +5254,10 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>111</v>
       </c>
       <c r="B5">
-        <f>'Table MV-1'!D13/'Table MV-1'!$D$61</f>
-        <v>8.298230946218824E-3</v>
+        <v>0</v>
       </c>
       <c r="C5">
         <f>'Table MV-1'!G13/'Table MV-1'!$G$61</f>
@@ -5136,11 +5279,10 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="B6">
-        <f>'Table MV-1'!D14/'Table MV-1'!$D$61</f>
-        <v>0.13507737172957132</v>
+        <v>0</v>
       </c>
       <c r="C6">
         <f>'Table MV-1'!G14/'Table MV-1'!$G$61</f>
@@ -5162,11 +5304,10 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="B7">
-        <f>'Table MV-1'!D15/'Table MV-1'!$D$61</f>
-        <v>1.5589702031572649E-2</v>
+        <v>0</v>
       </c>
       <c r="C7">
         <f>'Table MV-1'!G15/'Table MV-1'!$G$61</f>
@@ -5188,11 +5329,10 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>114</v>
       </c>
       <c r="B8">
-        <f>'Table MV-1'!D16/'Table MV-1'!$D$61</f>
-        <v>1.1520117410612801E-2</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <f>'Table MV-1'!G16/'Table MV-1'!$G$61</f>
@@ -5214,11 +5354,10 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>115</v>
       </c>
       <c r="B9">
-        <f>'Table MV-1'!D17/'Table MV-1'!$D$61</f>
-        <v>3.955997652548668E-3</v>
+        <v>0</v>
       </c>
       <c r="C9">
         <f>'Table MV-1'!G17/'Table MV-1'!$G$61</f>
@@ -5240,11 +5379,10 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="B10">
-        <f>'Table MV-1'!D18/'Table MV-1'!$D$61</f>
-        <v>2.0002511050046939E-3</v>
+        <v>0</v>
       </c>
       <c r="C10">
         <f>'Table MV-1'!G18/'Table MV-1'!$G$61</f>
@@ -5266,11 +5404,10 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>117</v>
       </c>
       <c r="B11">
-        <f>'Table MV-1'!D19/'Table MV-1'!$D$61</f>
-        <v>7.4585348593669304E-2</v>
+        <v>0</v>
       </c>
       <c r="C11">
         <f>'Table MV-1'!G19/'Table MV-1'!$G$61</f>
@@ -5292,11 +5429,10 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>118</v>
       </c>
       <c r="B12">
-        <f>'Table MV-1'!D20/'Table MV-1'!$D$61</f>
-        <v>3.3246882826224872E-2</v>
+        <v>0</v>
       </c>
       <c r="C12">
         <f>'Table MV-1'!G20/'Table MV-1'!$G$61</f>
@@ -5318,11 +5454,10 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>119</v>
       </c>
       <c r="B13">
-        <f>'Table MV-1'!D21/'Table MV-1'!$D$61</f>
-        <v>4.5177880312321358E-3</v>
+        <v>0</v>
       </c>
       <c r="C13">
         <f>'Table MV-1'!G21/'Table MV-1'!$G$61</f>
@@ -5344,11 +5479,10 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>120</v>
       </c>
       <c r="B14">
-        <f>'Table MV-1'!D22/'Table MV-1'!$D$61</f>
-        <v>5.5962364686266176E-3</v>
+        <v>0</v>
       </c>
       <c r="C14">
         <f>'Table MV-1'!G22/'Table MV-1'!$G$61</f>
@@ -5370,11 +5504,10 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>121</v>
       </c>
       <c r="B15">
-        <f>'Table MV-1'!D23/'Table MV-1'!$D$61</f>
-        <v>3.9583802966272987E-2</v>
+        <v>0</v>
       </c>
       <c r="C15">
         <f>'Table MV-1'!G23/'Table MV-1'!$G$61</f>
@@ -5396,11 +5529,10 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>122</v>
       </c>
       <c r="B16">
-        <f>'Table MV-1'!D24/'Table MV-1'!$D$61</f>
-        <v>2.0200142102604929E-2</v>
+        <v>0</v>
       </c>
       <c r="C16">
         <f>'Table MV-1'!G24/'Table MV-1'!$G$61</f>
@@ -5422,11 +5554,10 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>123</v>
       </c>
       <c r="B17">
-        <f>'Table MV-1'!D25/'Table MV-1'!$D$61</f>
-        <v>1.1069079557484499E-2</v>
+        <v>0</v>
       </c>
       <c r="C17">
         <f>'Table MV-1'!G25/'Table MV-1'!$G$61</f>
@@ -5448,11 +5579,10 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>124</v>
       </c>
       <c r="B18">
-        <f>'Table MV-1'!D26/'Table MV-1'!$D$61</f>
-        <v>8.4565602609209273E-3</v>
+        <v>0</v>
       </c>
       <c r="C18">
         <f>'Table MV-1'!G26/'Table MV-1'!$G$61</f>
@@ -5474,11 +5604,10 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>125</v>
       </c>
       <c r="B19">
-        <f>'Table MV-1'!D27/'Table MV-1'!$D$61</f>
-        <v>1.5641720716067772E-2</v>
+        <v>0</v>
       </c>
       <c r="C19">
         <f>'Table MV-1'!G27/'Table MV-1'!$G$61</f>
@@ -5500,11 +5629,10 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>126</v>
       </c>
       <c r="B20">
-        <f>'Table MV-1'!D28/'Table MV-1'!$D$61</f>
-        <v>1.2514264951923855E-2</v>
+        <v>0</v>
       </c>
       <c r="C20">
         <f>'Table MV-1'!G28/'Table MV-1'!$G$61</f>
@@ -5526,11 +5654,10 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>127</v>
       </c>
       <c r="B21">
-        <f>'Table MV-1'!D29/'Table MV-1'!$D$61</f>
-        <v>3.3868643547885439E-3</v>
+        <v>0</v>
       </c>
       <c r="C21">
         <f>'Table MV-1'!G29/'Table MV-1'!$G$61</f>
@@ -5552,11 +5679,10 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>128</v>
       </c>
       <c r="B22">
-        <f>'Table MV-1'!D30/'Table MV-1'!$D$61</f>
-        <v>1.7344821387298082E-2</v>
+        <v>0</v>
       </c>
       <c r="C22">
         <f>'Table MV-1'!G30/'Table MV-1'!$G$61</f>
@@ -5578,11 +5704,10 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>83</v>
+        <v>129</v>
       </c>
       <c r="B23">
-        <f>'Table MV-1'!D31/'Table MV-1'!$D$61</f>
-        <v>1.9055188885179382E-2</v>
+        <v>0</v>
       </c>
       <c r="C23">
         <f>'Table MV-1'!G31/'Table MV-1'!$G$61</f>
@@ -5604,11 +5729,10 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>36</v>
+        <v>130</v>
       </c>
       <c r="B24">
-        <f>'Table MV-1'!D32/'Table MV-1'!$D$61</f>
-        <v>2.5602285816466973E-2</v>
+        <v>0</v>
       </c>
       <c r="C24">
         <f>'Table MV-1'!G32/'Table MV-1'!$G$61</f>
@@ -5630,11 +5754,10 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>131</v>
       </c>
       <c r="B25">
-        <f>'Table MV-1'!D33/'Table MV-1'!$D$61</f>
-        <v>1.7517332427833467E-2</v>
+        <v>0</v>
       </c>
       <c r="C25">
         <f>'Table MV-1'!G33/'Table MV-1'!$G$61</f>
@@ -5656,11 +5779,10 @@
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>132</v>
       </c>
       <c r="B26">
-        <f>'Table MV-1'!D34/'Table MV-1'!$D$61</f>
-        <v>7.4991463380995726E-3</v>
+        <v>0</v>
       </c>
       <c r="C26">
         <f>'Table MV-1'!G34/'Table MV-1'!$G$61</f>
@@ -5682,11 +5804,10 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="B27">
-        <f>'Table MV-1'!D35/'Table MV-1'!$D$61</f>
-        <v>1.8941078781341755E-2</v>
+        <v>0</v>
       </c>
       <c r="C27">
         <f>'Table MV-1'!G35/'Table MV-1'!$G$61</f>
@@ -5708,11 +5829,10 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>32</v>
+        <v>134</v>
       </c>
       <c r="B28">
-        <f>'Table MV-1'!D36/'Table MV-1'!$D$61</f>
-        <v>4.3665733583296952E-3</v>
+        <v>0</v>
       </c>
       <c r="C28">
         <f>'Table MV-1'!G36/'Table MV-1'!$G$61</f>
@@ -5734,11 +5854,10 @@
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>135</v>
       </c>
       <c r="B29">
-        <f>'Table MV-1'!D37/'Table MV-1'!$D$61</f>
-        <v>5.9438361806167864E-3</v>
+        <v>0</v>
       </c>
       <c r="C29">
         <f>'Table MV-1'!G37/'Table MV-1'!$G$61</f>
@@ -5760,11 +5879,10 @@
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>136</v>
       </c>
       <c r="B30">
-        <f>'Table MV-1'!D38/'Table MV-1'!$D$61</f>
-        <v>9.7731494559867137E-3</v>
+        <v>0</v>
       </c>
       <c r="C30">
         <f>'Table MV-1'!G38/'Table MV-1'!$G$61</f>
@@ -5786,11 +5904,10 @@
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="B31">
-        <f>'Table MV-1'!D39/'Table MV-1'!$D$61</f>
-        <v>4.3831615071246288E-3</v>
+        <v>0</v>
       </c>
       <c r="C31">
         <f>'Table MV-1'!G39/'Table MV-1'!$G$61</f>
@@ -5812,11 +5929,10 @@
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>138</v>
       </c>
       <c r="B32">
-        <f>'Table MV-1'!D40/'Table MV-1'!$D$61</f>
-        <v>2.4170045645943845E-2</v>
+        <v>0</v>
       </c>
       <c r="C32">
         <f>'Table MV-1'!G40/'Table MV-1'!$G$61</f>
@@ -5838,11 +5954,10 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>27</v>
+        <v>139</v>
       </c>
       <c r="B33">
-        <f>'Table MV-1'!D41/'Table MV-1'!$D$61</f>
-        <v>5.9347811819626707E-3</v>
+        <v>0</v>
       </c>
       <c r="C33">
         <f>'Table MV-1'!G41/'Table MV-1'!$G$61</f>
@@ -5864,11 +5979,10 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>26</v>
+        <v>140</v>
       </c>
       <c r="B34">
-        <f>'Table MV-1'!D42/'Table MV-1'!$D$61</f>
-        <v>4.0260007818496736E-2</v>
+        <v>0</v>
       </c>
       <c r="C34">
         <f>'Table MV-1'!G42/'Table MV-1'!$G$61</f>
@@ -5890,11 +6004,10 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>25</v>
+        <v>141</v>
       </c>
       <c r="B35">
-        <f>'Table MV-1'!D43/'Table MV-1'!$D$61</f>
-        <v>3.232472823114596E-2</v>
+        <v>0</v>
       </c>
       <c r="C35">
         <f>'Table MV-1'!G43/'Table MV-1'!$G$61</f>
@@ -5916,11 +6029,10 @@
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>24</v>
+        <v>142</v>
       </c>
       <c r="B36">
-        <f>'Table MV-1'!D44/'Table MV-1'!$D$61</f>
-        <v>2.0512044955405084E-3</v>
+        <v>0</v>
       </c>
       <c r="C36">
         <f>'Table MV-1'!G44/'Table MV-1'!$G$61</f>
@@ -5942,11 +6054,10 @@
     </row>
     <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>23</v>
+        <v>143</v>
       </c>
       <c r="B37">
-        <f>'Table MV-1'!D45/'Table MV-1'!$D$61</f>
-        <v>4.0403584714173067E-2</v>
+        <v>0</v>
       </c>
       <c r="C37">
         <f>'Table MV-1'!G45/'Table MV-1'!$G$61</f>
@@ -5968,11 +6079,10 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>22</v>
+        <v>144</v>
       </c>
       <c r="B38">
-        <f>'Table MV-1'!D46/'Table MV-1'!$D$61</f>
-        <v>1.1640695370631938E-2</v>
+        <v>0</v>
       </c>
       <c r="C38">
         <f>'Table MV-1'!G46/'Table MV-1'!$G$61</f>
@@ -5994,11 +6104,10 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>21</v>
+        <v>145</v>
       </c>
       <c r="B39">
-        <f>'Table MV-1'!D47/'Table MV-1'!$D$61</f>
-        <v>1.3704702416790554E-2</v>
+        <v>0</v>
       </c>
       <c r="C39">
         <f>'Table MV-1'!G47/'Table MV-1'!$G$61</f>
@@ -6020,11 +6129,10 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>146</v>
       </c>
       <c r="B40">
-        <f>'Table MV-1'!D48/'Table MV-1'!$D$61</f>
-        <v>3.846201038090917E-2</v>
+        <v>0</v>
       </c>
       <c r="C40">
         <f>'Table MV-1'!G48/'Table MV-1'!$G$61</f>
@@ -6046,11 +6154,10 @@
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>19</v>
+        <v>147</v>
       </c>
       <c r="B41">
-        <f>'Table MV-1'!D49/'Table MV-1'!$D$61</f>
-        <v>3.6311971335983252E-3</v>
+        <v>0</v>
       </c>
       <c r="C41">
         <f>'Table MV-1'!G49/'Table MV-1'!$G$61</f>
@@ -6072,11 +6179,10 @@
     </row>
     <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>18</v>
+        <v>148</v>
       </c>
       <c r="B42">
-        <f>'Table MV-1'!D50/'Table MV-1'!$D$61</f>
-        <v>1.6810224539236585E-2</v>
+        <v>0</v>
       </c>
       <c r="C42">
         <f>'Table MV-1'!G50/'Table MV-1'!$G$61</f>
@@ -6098,11 +6204,10 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>17</v>
+        <v>149</v>
       </c>
       <c r="B43">
-        <f>'Table MV-1'!D51/'Table MV-1'!$D$61</f>
-        <v>3.0912643041870807E-3</v>
+        <v>0</v>
       </c>
       <c r="C43">
         <f>'Table MV-1'!G51/'Table MV-1'!$G$61</f>
@@ -6124,11 +6229,10 @@
     </row>
     <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>16</v>
+        <v>150</v>
       </c>
       <c r="B44">
-        <f>'Table MV-1'!D52/'Table MV-1'!$D$61</f>
-        <v>2.0122946336767956E-2</v>
+        <v>0</v>
       </c>
       <c r="C44">
         <f>'Table MV-1'!G52/'Table MV-1'!$G$61</f>
@@ -6150,11 +6254,10 @@
     </row>
     <row r="45" spans="1:7">
       <c r="A45" t="s">
-        <v>15</v>
+        <v>151</v>
       </c>
       <c r="B45">
-        <f>'Table MV-1'!D53/'Table MV-1'!$D$61</f>
-        <v>7.6929994017233036E-2</v>
+        <v>0</v>
       </c>
       <c r="C45">
         <f>'Table MV-1'!G53/'Table MV-1'!$G$61</f>
@@ -6176,11 +6279,10 @@
     </row>
     <row r="46" spans="1:7">
       <c r="A46" t="s">
-        <v>14</v>
+        <v>152</v>
       </c>
       <c r="B46">
-        <f>'Table MV-1'!D54/'Table MV-1'!$D$61</f>
-        <v>8.5862978466794693E-3</v>
+        <v>0</v>
       </c>
       <c r="C46">
         <f>'Table MV-1'!G54/'Table MV-1'!$G$61</f>
@@ -6202,11 +6304,10 @@
     </row>
     <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>153</v>
       </c>
       <c r="B47">
-        <f>'Table MV-1'!D55/'Table MV-1'!$D$61</f>
-        <v>1.8396009713198137E-3</v>
+        <v>0</v>
       </c>
       <c r="C47">
         <f>'Table MV-1'!G55/'Table MV-1'!$G$61</f>
@@ -6228,11 +6329,10 @@
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>154</v>
       </c>
       <c r="B48">
-        <f>'Table MV-1'!D56/'Table MV-1'!$D$61</f>
-        <v>2.9079234091689471E-2</v>
+        <v>0</v>
       </c>
       <c r="C48">
         <f>'Table MV-1'!G56/'Table MV-1'!$G$61</f>
@@ -6254,11 +6354,10 @@
     </row>
     <row r="49" spans="1:7">
       <c r="A49" t="s">
-        <v>11</v>
+        <v>155</v>
       </c>
       <c r="B49">
-        <f>'Table MV-1'!D57/'Table MV-1'!$D$61</f>
-        <v>2.6635868257378827E-2</v>
+        <v>0</v>
       </c>
       <c r="C49">
         <f>'Table MV-1'!G57/'Table MV-1'!$G$61</f>
@@ -6280,11 +6379,10 @@
     </row>
     <row r="50" spans="1:7">
       <c r="A50" t="s">
-        <v>10</v>
+        <v>156</v>
       </c>
       <c r="B50">
-        <f>'Table MV-1'!D58/'Table MV-1'!$D$61</f>
-        <v>4.8381751894939189E-3</v>
+        <v>0</v>
       </c>
       <c r="C50">
         <f>'Table MV-1'!G58/'Table MV-1'!$G$61</f>
@@ -6306,11 +6404,10 @@
     </row>
     <row r="51" spans="1:7">
       <c r="A51" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="B51">
-        <f>'Table MV-1'!D59/'Table MV-1'!$D$61</f>
-        <v>1.8086189890550556E-2</v>
+        <v>0</v>
       </c>
       <c r="C51">
         <f>'Table MV-1'!G59/'Table MV-1'!$G$61</f>
@@ -6332,11 +6429,10 @@
     </row>
     <row r="52" spans="1:7">
       <c r="A52" t="s">
-        <v>8</v>
+        <v>158</v>
       </c>
       <c r="B52">
-        <f>'Table MV-1'!D60/'Table MV-1'!$D$61</f>
-        <v>1.8198644984129973E-3</v>
+        <v>0</v>
       </c>
       <c r="C52">
         <f>'Table MV-1'!G60/'Table MV-1'!$G$61</f>
@@ -6575,10 +6671,10 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:G61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="7" width="13.7109375" customWidth="1"/>
+    <col min="2" max="7" width="13.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">

</xml_diff>